<commit_message>
feat: UK dashboard, interactive calculator, refined responsive design
- Add UK region: ONS CPI fetcher (D7BT, 2015=100), GBP, 37.5 h/week
- Refactor pipeline as multi-region (src/regions.py)
- Interactive calculator: visitors plug in their own salary, hours, base year and CPI month — live recalc
- Cross-region nav: 🇨🇭 Switzerland ⇄ 🇬🇧 UK
- Refined design: Inter font, dark-mode aware, smoother breakpoints, touch-friendly inputs, tabular numbers, hover lift on cards
- Region-aware Excel + processed CSV outputs (per region)

Documented assumptions:
- UK working hours: 37.5/week × 52 = 1,950 h/year (standard full-time)
- UK salary placeholder: £45k → £50k 2023→2026 (edit salary_inputs_uk.csv)
- UK CPI base: 2015 = 100, ONS series D7BT

https://claude.ai/code/session_01LoVHdtpynSkP9unNWSRc8c
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker.xlsx
+++ b/data/processed/salary_tracker.xlsx
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3379,120 +3379,130 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>current_salary_year</t>
+          <t>weekly_hours</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2026</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nominal_monthly</t>
+          <t>current_salary_year</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8100</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nominal_annual</t>
+          <t>nominal_monthly</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>105300</v>
+        <v>8100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>nominal_hourly</t>
+          <t>nominal_annual</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48.21</v>
+        <v>105300</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>real_monthly</t>
+          <t>nominal_hourly</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8026.74</v>
+        <v>48.21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>real_annual</t>
+          <t>real_monthly</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>104347.67</v>
+        <v>8026.74</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>real_hourly</t>
+          <t>real_annual</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>47.78</v>
+        <v>104347.67</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cumulative_inflation_pct</t>
+          <t>real_hourly</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.91</v>
+        <v>47.78</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>nominal_increase_vs_base_pct</t>
+          <t>cumulative_inflation_pct</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10.96</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>real_increase_vs_base_pct</t>
+          <t>nominal_increase_vs_base_pct</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9.960000000000001</v>
+        <v>10.96</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>annual_gain_loss_vs_base</t>
+          <t>real_increase_vs_base_pct</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9447.67</v>
+        <v>9.960000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>annual_gain_loss_vs_base</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9447.67</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>monthly_gain_loss_vs_base</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B19" t="n">
         <v>726.74</v>
       </c>
     </row>

</xml_diff>